<commit_message>
Rename donor cards to match kvittel spelling: Yosef, Zev, Netaniel
Per request, set the Hebrew first names on the cards to the kvittel spelling
(יוסי→יוסף גולדבורד, זאבי→זאב שטרן, נתנאל→נתניאל דואק); old spelling kept
as an alias. Prayers now link by exact name.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -7271,7 +7271,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>יוסי</t>
+          <t>יוסף</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -7343,7 +7343,11 @@
       <c r="R102" s="2" t="inlineStr"/>
       <c r="S102" s="2" t="inlineStr"/>
       <c r="T102" s="2" t="inlineStr"/>
-      <c r="U102" s="2" t="inlineStr"/>
+      <c r="U102" s="2" t="inlineStr">
+        <is>
+          <t>יוסי</t>
+        </is>
+      </c>
       <c r="V102" s="2" t="inlineStr">
         <is>
           <t>ppppppp-----</t>
@@ -10397,7 +10401,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>נתנאל</t>
+          <t>נתניאל</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -10473,7 +10477,11 @@
           <t>מוזג מכפילות</t>
         </is>
       </c>
-      <c r="U152" s="2" t="inlineStr"/>
+      <c r="U152" s="2" t="inlineStr">
+        <is>
+          <t>נתנאל</t>
+        </is>
+      </c>
       <c r="V152" s="2" t="inlineStr">
         <is>
           <t>ppppppp-----</t>
@@ -35774,7 +35782,7 @@
       </c>
       <c r="C547" s="2" t="inlineStr">
         <is>
-          <t>זאבי</t>
+          <t>זאב</t>
         </is>
       </c>
       <c r="D547" s="2" t="inlineStr">
@@ -35846,7 +35854,11 @@
       <c r="R547" s="2" t="inlineStr"/>
       <c r="S547" s="2" t="inlineStr"/>
       <c r="T547" s="2" t="inlineStr"/>
-      <c r="U547" s="2" t="inlineStr"/>
+      <c r="U547" s="2" t="inlineStr">
+        <is>
+          <t>זאבי</t>
+        </is>
+      </c>
       <c r="V547" s="2" t="inlineStr">
         <is>
           <t>ppppppp-----</t>

</xml_diff>

<commit_message>
Backfill 12 missing phone numbers from exact-name Google contacts
Some donors had an empty phone even though their own Google Contacts entry
carried valid numbers (the pipeline only read Phone 1/2 of the matched
duplicate). Enrich empty phone fields from the exact same-name contact across
all phone columns, normalized and de-duplicated. Family-only (same-surname)
matches are intentionally left untouched to avoid wrong attributions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -1253,7 +1253,11 @@
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>+972 548455419</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
@@ -3873,7 +3877,11 @@
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>+1 347-985-3263</t>
+        </is>
+      </c>
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
@@ -4718,7 +4726,11 @@
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-613-0102</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
@@ -5741,7 +5753,11 @@
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>+1 374-541-3163 / +1 347-541-3163 / +1 917-498-2555 / +1 914-314-8421</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
@@ -12472,7 +12488,11 @@
       </c>
       <c r="D182" s="2" t="inlineStr"/>
       <c r="E182" s="2" t="inlineStr"/>
-      <c r="F182" s="2" t="inlineStr"/>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-836-0609 / +1 212-362-5643 / +1 212-362-8807</t>
+        </is>
+      </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
           <t>mhalpern12@gmail.com</t>
@@ -15007,7 +15027,11 @@
       </c>
       <c r="D222" s="2" t="inlineStr"/>
       <c r="E222" s="2" t="inlineStr"/>
-      <c r="F222" s="2" t="inlineStr"/>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>+1 732-824-1456</t>
+        </is>
+      </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
           <t>Eweingarden@gmail.com</t>
@@ -15572,7 +15596,11 @@
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr"/>
-      <c r="F231" s="2" t="inlineStr"/>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-974-1750</t>
+        </is>
+      </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
           <t>msilber@silberlawny.com</t>
@@ -21295,7 +21323,11 @@
       </c>
       <c r="D320" s="2" t="inlineStr"/>
       <c r="E320" s="2" t="inlineStr"/>
-      <c r="F320" s="2" t="inlineStr"/>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>+1 732-575-3142</t>
+        </is>
+      </c>
       <c r="G320" s="2" t="inlineStr"/>
       <c r="H320" s="2" t="inlineStr"/>
       <c r="I320" s="2" t="inlineStr"/>
@@ -31227,7 +31259,11 @@
         </is>
       </c>
       <c r="E472" s="2" t="inlineStr"/>
-      <c r="F472" s="2" t="inlineStr"/>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-377-2571 / +1 917-597-3775</t>
+        </is>
+      </c>
       <c r="G472" s="2" t="inlineStr">
         <is>
           <t>mkohn@mfandco.com</t>
@@ -33402,7 +33438,11 @@
       </c>
       <c r="D507" s="2" t="inlineStr"/>
       <c r="E507" s="2" t="inlineStr"/>
-      <c r="F507" s="2" t="inlineStr"/>
+      <c r="F507" s="2" t="inlineStr">
+        <is>
+          <t>+972 533158007</t>
+        </is>
+      </c>
       <c r="G507" s="2" t="inlineStr"/>
       <c r="H507" s="2" t="inlineStr"/>
       <c r="I507" s="2" t="inlineStr"/>
@@ -34595,7 +34635,11 @@
         </is>
       </c>
       <c r="E527" s="2" t="inlineStr"/>
-      <c r="F527" s="2" t="inlineStr"/>
+      <c r="F527" s="2" t="inlineStr">
+        <is>
+          <t>+1 514-652-1926</t>
+        </is>
+      </c>
       <c r="G527" s="2" t="inlineStr">
         <is>
           <t>mikelive5@hotmail.com</t>
@@ -36775,7 +36819,11 @@
       </c>
       <c r="D563" s="2" t="inlineStr"/>
       <c r="E563" s="2" t="inlineStr"/>
-      <c r="F563" s="2" t="inlineStr"/>
+      <c r="F563" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-416-0228</t>
+        </is>
+      </c>
       <c r="G563" s="2" t="inlineStr">
         <is>
           <t>mike@schondevelopment.com</t>

</xml_diff>

<commit_message>
Attach Abramowitz phones; backfill 28 phones from same-surname relatives
- Elchanan Abramowitz: attach the two numbers filed under "ב.אברמוביץ"
  (confirmed same person); keep that spelling as an alias.
- Fill empty phones from a same-surname Google contact only when unambiguous
  (<=2 distinct numbers for that surname). Common surnames with many differing
  numbers (Friedman, Klein, Katz...) are left blank rather than risk a wrong one.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -681,7 +681,11 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-377-0930 / +1 718-677-6869</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>elchanan@sterlingwm.com</t>
@@ -740,7 +744,11 @@
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>ב.אברמוביץ</t>
+        </is>
+      </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
           <t>ppppppp-----</t>
@@ -2099,7 +2107,11 @@
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>+972 533811989 / +1 908-330-9001</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
@@ -2749,7 +2761,11 @@
       </c>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>+1 347-482-5177 / +1 917-686-9833</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
           <t>esti4gutman@yahoo.com</t>
@@ -2794,7 +2810,11 @@
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-809-6928 / +972 584052157</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>effiinwili@gmail.com</t>
@@ -5611,7 +5631,11 @@
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-754-6634</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>sbrody11211@yahoo.com</t>
@@ -12045,7 +12069,11 @@
       </c>
       <c r="D175" s="2" t="inlineStr"/>
       <c r="E175" s="2" t="inlineStr"/>
-      <c r="F175" s="2" t="inlineStr"/>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>+972 542615474</t>
+        </is>
+      </c>
       <c r="G175" s="2" t="inlineStr"/>
       <c r="H175" s="2" t="inlineStr"/>
       <c r="I175" s="2" t="inlineStr"/>
@@ -13961,7 +13989,11 @@
       </c>
       <c r="D203" s="2" t="inlineStr"/>
       <c r="E203" s="2" t="inlineStr"/>
-      <c r="F203" s="2" t="inlineStr"/>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>+1 732-664-1000</t>
+        </is>
+      </c>
       <c r="G203" s="2" t="inlineStr"/>
       <c r="H203" s="2" t="inlineStr"/>
       <c r="I203" s="2" t="inlineStr"/>
@@ -14290,7 +14322,11 @@
       </c>
       <c r="D208" s="2" t="inlineStr"/>
       <c r="E208" s="2" t="inlineStr"/>
-      <c r="F208" s="2" t="inlineStr"/>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>+1 347-243-1500</t>
+        </is>
+      </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
           <t>simonw11204@gmail.com</t>
@@ -15681,7 +15717,11 @@
       </c>
       <c r="D232" s="2" t="inlineStr"/>
       <c r="E232" s="2" t="inlineStr"/>
-      <c r="F232" s="2" t="inlineStr"/>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>+972 548679292 / +972 527319882</t>
+        </is>
+      </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
           <t>michaelsinger@live.com.au</t>
@@ -15831,7 +15871,11 @@
       </c>
       <c r="D234" s="2" t="inlineStr"/>
       <c r="E234" s="2" t="inlineStr"/>
-      <c r="F234" s="2" t="inlineStr"/>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>+972 527168435</t>
+        </is>
+      </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
           <t>david@britanniagroup.NYC</t>
@@ -16088,7 +16132,11 @@
       </c>
       <c r="D239" s="2" t="inlineStr"/>
       <c r="E239" s="2" t="inlineStr"/>
-      <c r="F239" s="2" t="inlineStr"/>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-929-6162</t>
+        </is>
+      </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
           <t>etabak@bluestonegrp.com</t>
@@ -16984,7 +17032,11 @@
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr"/>
-      <c r="F251" s="2" t="inlineStr"/>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>01312019883095</t>
+        </is>
+      </c>
       <c r="G251" s="2" t="inlineStr"/>
       <c r="H251" s="2" t="inlineStr"/>
       <c r="I251" s="2" t="inlineStr">
@@ -17829,7 +17881,11 @@
       </c>
       <c r="D264" s="2" t="inlineStr"/>
       <c r="E264" s="2" t="inlineStr"/>
-      <c r="F264" s="2" t="inlineStr"/>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>+972 539356249 / +1 516-791-3311</t>
+        </is>
+      </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
           <t>lisajacobson11@gmail.com</t>
@@ -21680,7 +21736,11 @@
       </c>
       <c r="D325" s="2" t="inlineStr"/>
       <c r="E325" s="2" t="inlineStr"/>
-      <c r="F325" s="2" t="inlineStr"/>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>44 161 773 3670 / 07904-281848</t>
+        </is>
+      </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
           <t>smusic@talktalk.net</t>
@@ -22051,7 +22111,11 @@
       </c>
       <c r="D332" s="2" t="inlineStr"/>
       <c r="E332" s="2" t="inlineStr"/>
-      <c r="F332" s="2" t="inlineStr"/>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-261-3446 / +1 516-610-5047</t>
+        </is>
+      </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
           <t>mmmoscovitz@gmail.com</t>
@@ -23909,7 +23973,11 @@
       </c>
       <c r="D358" s="2" t="inlineStr"/>
       <c r="E358" s="2" t="inlineStr"/>
-      <c r="F358" s="2" t="inlineStr"/>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>+1 732-267-6746</t>
+        </is>
+      </c>
       <c r="G358" s="2" t="inlineStr"/>
       <c r="H358" s="2" t="inlineStr"/>
       <c r="I358" s="2" t="inlineStr"/>
@@ -24295,7 +24363,11 @@
       </c>
       <c r="D364" s="2" t="inlineStr"/>
       <c r="E364" s="2" t="inlineStr"/>
-      <c r="F364" s="2" t="inlineStr"/>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>+1 732-523-1113</t>
+        </is>
+      </c>
       <c r="G364" s="2" t="inlineStr">
         <is>
           <t>33miron@gmail.com</t>
@@ -24446,7 +24518,11 @@
       </c>
       <c r="D367" s="2" t="inlineStr"/>
       <c r="E367" s="2" t="inlineStr"/>
-      <c r="F367" s="2" t="inlineStr"/>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-339-2468</t>
+        </is>
+      </c>
       <c r="G367" s="2" t="inlineStr">
         <is>
           <t>Rivky.Nussbaum@lsdco.com</t>
@@ -28767,7 +28843,11 @@
       </c>
       <c r="D432" s="2" t="inlineStr"/>
       <c r="E432" s="2" t="inlineStr"/>
-      <c r="F432" s="2" t="inlineStr"/>
+      <c r="F432" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-501-8806</t>
+        </is>
+      </c>
       <c r="G432" s="2" t="inlineStr">
         <is>
           <t>df@thelesergroup.com</t>
@@ -29331,7 +29411,11 @@
       </c>
       <c r="D440" s="2" t="inlineStr"/>
       <c r="E440" s="2" t="inlineStr"/>
-      <c r="F440" s="2" t="inlineStr"/>
+      <c r="F440" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-471-1626</t>
+        </is>
+      </c>
       <c r="G440" s="2" t="inlineStr">
         <is>
           <t>Fertig.Y@fibi.co.il</t>
@@ -30104,7 +30188,11 @@
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr"/>
-      <c r="F453" s="2" t="inlineStr"/>
+      <c r="F453" s="2" t="inlineStr">
+        <is>
+          <t>+1 516-295-3181 / +1 516-633-3548</t>
+        </is>
+      </c>
       <c r="G453" s="2" t="inlineStr"/>
       <c r="H453" s="2" t="inlineStr"/>
       <c r="I453" s="2" t="inlineStr">
@@ -31624,7 +31712,11 @@
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr"/>
-      <c r="F477" s="2" t="inlineStr"/>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>+1 650-703-1237</t>
+        </is>
+      </c>
       <c r="G477" s="2" t="inlineStr">
         <is>
           <t>esti.karp@gmail.com</t>
@@ -32217,7 +32309,11 @@
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr"/>
-      <c r="F486" s="2" t="inlineStr"/>
+      <c r="F486" s="2" t="inlineStr">
+        <is>
+          <t>+1 917-209-5919</t>
+        </is>
+      </c>
       <c r="G486" s="2" t="inlineStr"/>
       <c r="H486" s="2" t="inlineStr"/>
       <c r="I486" s="2" t="inlineStr">
@@ -33601,7 +33697,11 @@
       </c>
       <c r="D510" s="2" t="inlineStr"/>
       <c r="E510" s="2" t="inlineStr"/>
-      <c r="F510" s="2" t="inlineStr"/>
+      <c r="F510" s="2" t="inlineStr">
+        <is>
+          <t>+972 556686050</t>
+        </is>
+      </c>
       <c r="G510" s="2" t="inlineStr">
         <is>
           <t>chanirubenstein@gmail.com</t>
@@ -33707,7 +33807,11 @@
       </c>
       <c r="D512" s="2" t="inlineStr"/>
       <c r="E512" s="2" t="inlineStr"/>
-      <c r="F512" s="2" t="inlineStr"/>
+      <c r="F512" s="2" t="inlineStr">
+        <is>
+          <t>+1 914-806-5826</t>
+        </is>
+      </c>
       <c r="G512" s="2" t="inlineStr">
         <is>
           <t>deenadee94@gmail.com</t>
@@ -34805,7 +34909,11 @@
       </c>
       <c r="D529" s="2" t="inlineStr"/>
       <c r="E529" s="2" t="inlineStr"/>
-      <c r="F529" s="2" t="inlineStr"/>
+      <c r="F529" s="2" t="inlineStr">
+        <is>
+          <t>+380633855610</t>
+        </is>
+      </c>
       <c r="G529" s="2" t="inlineStr">
         <is>
           <t>charles.rappaport@gmail.com</t>
@@ -34903,7 +35011,11 @@
       </c>
       <c r="D531" s="2" t="inlineStr"/>
       <c r="E531" s="2" t="inlineStr"/>
-      <c r="F531" s="2" t="inlineStr"/>
+      <c r="F531" s="2" t="inlineStr">
+        <is>
+          <t>+972 586188883</t>
+        </is>
+      </c>
       <c r="G531" s="2" t="inlineStr">
         <is>
           <t>pinishaool@gmail.com</t>
@@ -35013,7 +35125,11 @@
       </c>
       <c r="D533" s="2" t="inlineStr"/>
       <c r="E533" s="2" t="inlineStr"/>
-      <c r="F533" s="2" t="inlineStr"/>
+      <c r="F533" s="2" t="inlineStr">
+        <is>
+          <t>+1 718-664-8508 / +1 646-261-7569</t>
+        </is>
+      </c>
       <c r="G533" s="2" t="inlineStr">
         <is>
           <t>baruchsebat@gmail.com</t>
@@ -36729,7 +36845,11 @@
       </c>
       <c r="D561" s="2" t="inlineStr"/>
       <c r="E561" s="2" t="inlineStr"/>
-      <c r="F561" s="2" t="inlineStr"/>
+      <c r="F561" s="2" t="inlineStr">
+        <is>
+          <t>+972 504123124</t>
+        </is>
+      </c>
       <c r="G561" s="2" t="inlineStr">
         <is>
           <t>ronit030292@gmail.com</t>

</xml_diff>

<commit_message>
Add phone-verification web page; revert unconfirmed family phone fills
The bulk same-surname phone fills were not reliable enough to apply blindly, so
clear them and instead let the user confirm each. New /review-phones.html reads
phone_suggestions.json (donor + candidate number + source contact, sorted by
confidence) and applies an approved number via PUT /api/donor. Exact-name and
Abramowitz fixes are kept.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -2107,11 +2107,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>+972 533811989 / +1 908-330-9001</t>
-        </is>
-      </c>
+      <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
@@ -5631,11 +5627,7 @@
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>+1 917-754-6634</t>
-        </is>
-      </c>
+      <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>sbrody11211@yahoo.com</t>
@@ -12069,11 +12061,7 @@
       </c>
       <c r="D175" s="2" t="inlineStr"/>
       <c r="E175" s="2" t="inlineStr"/>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>+972 542615474</t>
-        </is>
-      </c>
+      <c r="F175" s="2" t="inlineStr"/>
       <c r="G175" s="2" t="inlineStr"/>
       <c r="H175" s="2" t="inlineStr"/>
       <c r="I175" s="2" t="inlineStr"/>
@@ -13989,11 +13977,7 @@
       </c>
       <c r="D203" s="2" t="inlineStr"/>
       <c r="E203" s="2" t="inlineStr"/>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>+1 732-664-1000</t>
-        </is>
-      </c>
+      <c r="F203" s="2" t="inlineStr"/>
       <c r="G203" s="2" t="inlineStr"/>
       <c r="H203" s="2" t="inlineStr"/>
       <c r="I203" s="2" t="inlineStr"/>
@@ -14322,11 +14306,7 @@
       </c>
       <c r="D208" s="2" t="inlineStr"/>
       <c r="E208" s="2" t="inlineStr"/>
-      <c r="F208" s="2" t="inlineStr">
-        <is>
-          <t>+1 347-243-1500</t>
-        </is>
-      </c>
+      <c r="F208" s="2" t="inlineStr"/>
       <c r="G208" s="2" t="inlineStr">
         <is>
           <t>simonw11204@gmail.com</t>
@@ -15717,11 +15697,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr"/>
       <c r="E232" s="2" t="inlineStr"/>
-      <c r="F232" s="2" t="inlineStr">
-        <is>
-          <t>+972 548679292 / +972 527319882</t>
-        </is>
-      </c>
+      <c r="F232" s="2" t="inlineStr"/>
       <c r="G232" s="2" t="inlineStr">
         <is>
           <t>michaelsinger@live.com.au</t>
@@ -15871,11 +15847,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr"/>
       <c r="E234" s="2" t="inlineStr"/>
-      <c r="F234" s="2" t="inlineStr">
-        <is>
-          <t>+972 527168435</t>
-        </is>
-      </c>
+      <c r="F234" s="2" t="inlineStr"/>
       <c r="G234" s="2" t="inlineStr">
         <is>
           <t>david@britanniagroup.NYC</t>
@@ -16132,11 +16104,7 @@
       </c>
       <c r="D239" s="2" t="inlineStr"/>
       <c r="E239" s="2" t="inlineStr"/>
-      <c r="F239" s="2" t="inlineStr">
-        <is>
-          <t>+1 917-929-6162</t>
-        </is>
-      </c>
+      <c r="F239" s="2" t="inlineStr"/>
       <c r="G239" s="2" t="inlineStr">
         <is>
           <t>etabak@bluestonegrp.com</t>
@@ -17032,11 +17000,7 @@
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr"/>
-      <c r="F251" s="2" t="inlineStr">
-        <is>
-          <t>01312019883095</t>
-        </is>
-      </c>
+      <c r="F251" s="2" t="inlineStr"/>
       <c r="G251" s="2" t="inlineStr"/>
       <c r="H251" s="2" t="inlineStr"/>
       <c r="I251" s="2" t="inlineStr">
@@ -17881,11 +17845,7 @@
       </c>
       <c r="D264" s="2" t="inlineStr"/>
       <c r="E264" s="2" t="inlineStr"/>
-      <c r="F264" s="2" t="inlineStr">
-        <is>
-          <t>+972 539356249 / +1 516-791-3311</t>
-        </is>
-      </c>
+      <c r="F264" s="2" t="inlineStr"/>
       <c r="G264" s="2" t="inlineStr">
         <is>
           <t>lisajacobson11@gmail.com</t>
@@ -21736,11 +21696,7 @@
       </c>
       <c r="D325" s="2" t="inlineStr"/>
       <c r="E325" s="2" t="inlineStr"/>
-      <c r="F325" s="2" t="inlineStr">
-        <is>
-          <t>44 161 773 3670 / 07904-281848</t>
-        </is>
-      </c>
+      <c r="F325" s="2" t="inlineStr"/>
       <c r="G325" s="2" t="inlineStr">
         <is>
           <t>smusic@talktalk.net</t>
@@ -22111,11 +22067,7 @@
       </c>
       <c r="D332" s="2" t="inlineStr"/>
       <c r="E332" s="2" t="inlineStr"/>
-      <c r="F332" s="2" t="inlineStr">
-        <is>
-          <t>+1 718-261-3446 / +1 516-610-5047</t>
-        </is>
-      </c>
+      <c r="F332" s="2" t="inlineStr"/>
       <c r="G332" s="2" t="inlineStr">
         <is>
           <t>mmmoscovitz@gmail.com</t>
@@ -23973,11 +23925,7 @@
       </c>
       <c r="D358" s="2" t="inlineStr"/>
       <c r="E358" s="2" t="inlineStr"/>
-      <c r="F358" s="2" t="inlineStr">
-        <is>
-          <t>+1 732-267-6746</t>
-        </is>
-      </c>
+      <c r="F358" s="2" t="inlineStr"/>
       <c r="G358" s="2" t="inlineStr"/>
       <c r="H358" s="2" t="inlineStr"/>
       <c r="I358" s="2" t="inlineStr"/>
@@ -24363,11 +24311,7 @@
       </c>
       <c r="D364" s="2" t="inlineStr"/>
       <c r="E364" s="2" t="inlineStr"/>
-      <c r="F364" s="2" t="inlineStr">
-        <is>
-          <t>+1 732-523-1113</t>
-        </is>
-      </c>
+      <c r="F364" s="2" t="inlineStr"/>
       <c r="G364" s="2" t="inlineStr">
         <is>
           <t>33miron@gmail.com</t>
@@ -24518,11 +24462,7 @@
       </c>
       <c r="D367" s="2" t="inlineStr"/>
       <c r="E367" s="2" t="inlineStr"/>
-      <c r="F367" s="2" t="inlineStr">
-        <is>
-          <t>+1 718-339-2468</t>
-        </is>
-      </c>
+      <c r="F367" s="2" t="inlineStr"/>
       <c r="G367" s="2" t="inlineStr">
         <is>
           <t>Rivky.Nussbaum@lsdco.com</t>
@@ -28843,11 +28783,7 @@
       </c>
       <c r="D432" s="2" t="inlineStr"/>
       <c r="E432" s="2" t="inlineStr"/>
-      <c r="F432" s="2" t="inlineStr">
-        <is>
-          <t>+1 917-501-8806</t>
-        </is>
-      </c>
+      <c r="F432" s="2" t="inlineStr"/>
       <c r="G432" s="2" t="inlineStr">
         <is>
           <t>df@thelesergroup.com</t>
@@ -29411,11 +29347,7 @@
       </c>
       <c r="D440" s="2" t="inlineStr"/>
       <c r="E440" s="2" t="inlineStr"/>
-      <c r="F440" s="2" t="inlineStr">
-        <is>
-          <t>+1 718-471-1626</t>
-        </is>
-      </c>
+      <c r="F440" s="2" t="inlineStr"/>
       <c r="G440" s="2" t="inlineStr">
         <is>
           <t>Fertig.Y@fibi.co.il</t>
@@ -30188,11 +30120,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr"/>
-      <c r="F453" s="2" t="inlineStr">
-        <is>
-          <t>+1 516-295-3181 / +1 516-633-3548</t>
-        </is>
-      </c>
+      <c r="F453" s="2" t="inlineStr"/>
       <c r="G453" s="2" t="inlineStr"/>
       <c r="H453" s="2" t="inlineStr"/>
       <c r="I453" s="2" t="inlineStr">
@@ -31712,11 +31640,7 @@
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr"/>
-      <c r="F477" s="2" t="inlineStr">
-        <is>
-          <t>+1 650-703-1237</t>
-        </is>
-      </c>
+      <c r="F477" s="2" t="inlineStr"/>
       <c r="G477" s="2" t="inlineStr">
         <is>
           <t>esti.karp@gmail.com</t>
@@ -32309,11 +32233,7 @@
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr"/>
-      <c r="F486" s="2" t="inlineStr">
-        <is>
-          <t>+1 917-209-5919</t>
-        </is>
-      </c>
+      <c r="F486" s="2" t="inlineStr"/>
       <c r="G486" s="2" t="inlineStr"/>
       <c r="H486" s="2" t="inlineStr"/>
       <c r="I486" s="2" t="inlineStr">
@@ -33697,11 +33617,7 @@
       </c>
       <c r="D510" s="2" t="inlineStr"/>
       <c r="E510" s="2" t="inlineStr"/>
-      <c r="F510" s="2" t="inlineStr">
-        <is>
-          <t>+972 556686050</t>
-        </is>
-      </c>
+      <c r="F510" s="2" t="inlineStr"/>
       <c r="G510" s="2" t="inlineStr">
         <is>
           <t>chanirubenstein@gmail.com</t>
@@ -33807,11 +33723,7 @@
       </c>
       <c r="D512" s="2" t="inlineStr"/>
       <c r="E512" s="2" t="inlineStr"/>
-      <c r="F512" s="2" t="inlineStr">
-        <is>
-          <t>+1 914-806-5826</t>
-        </is>
-      </c>
+      <c r="F512" s="2" t="inlineStr"/>
       <c r="G512" s="2" t="inlineStr">
         <is>
           <t>deenadee94@gmail.com</t>
@@ -34909,11 +34821,7 @@
       </c>
       <c r="D529" s="2" t="inlineStr"/>
       <c r="E529" s="2" t="inlineStr"/>
-      <c r="F529" s="2" t="inlineStr">
-        <is>
-          <t>+380633855610</t>
-        </is>
-      </c>
+      <c r="F529" s="2" t="inlineStr"/>
       <c r="G529" s="2" t="inlineStr">
         <is>
           <t>charles.rappaport@gmail.com</t>
@@ -35011,11 +34919,7 @@
       </c>
       <c r="D531" s="2" t="inlineStr"/>
       <c r="E531" s="2" t="inlineStr"/>
-      <c r="F531" s="2" t="inlineStr">
-        <is>
-          <t>+972 586188883</t>
-        </is>
-      </c>
+      <c r="F531" s="2" t="inlineStr"/>
       <c r="G531" s="2" t="inlineStr">
         <is>
           <t>pinishaool@gmail.com</t>
@@ -35125,11 +35029,7 @@
       </c>
       <c r="D533" s="2" t="inlineStr"/>
       <c r="E533" s="2" t="inlineStr"/>
-      <c r="F533" s="2" t="inlineStr">
-        <is>
-          <t>+1 718-664-8508 / +1 646-261-7569</t>
-        </is>
-      </c>
+      <c r="F533" s="2" t="inlineStr"/>
       <c r="G533" s="2" t="inlineStr">
         <is>
           <t>baruchsebat@gmail.com</t>
@@ -36845,11 +36745,7 @@
       </c>
       <c r="D561" s="2" t="inlineStr"/>
       <c r="E561" s="2" t="inlineStr"/>
-      <c r="F561" s="2" t="inlineStr">
-        <is>
-          <t>+972 504123124</t>
-        </is>
-      </c>
+      <c r="F561" s="2" t="inlineStr"/>
       <c r="G561" s="2" t="inlineStr">
         <is>
           <t>ronit030292@gmail.com</t>

</xml_diff>

<commit_message>
Remove 'קבועים' filter; stop tiered donors showing under מזדמנים
- Drop the קבועים chip from the main catalog per request.
- מזדמנים now means category=מזדמן AND no kvittel tier, so a tiered donor
  (e.g. Zev Lam, Yissachar-Zevulun) no longer appears in both places.
- Data: 7 donors that had a tier but were mislabeled מזדמן are set to קבוע;
  Zev Lam's monthly amount corrected 1500 -> 1000.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -7938,7 +7938,7 @@
       <c r="H111" s="2" t="inlineStr"/>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
@@ -12314,7 +12314,7 @@
       <c r="H179" s="2" t="inlineStr"/>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr"/>
@@ -18983,13 +18983,13 @@
       <c r="H281" s="2" t="inlineStr"/>
       <c r="I281" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr"/>
       <c r="K281" s="2" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="L281" s="2" t="inlineStr"/>
@@ -19658,7 +19658,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr"/>
@@ -22129,7 +22129,7 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr"/>
@@ -25955,7 +25955,7 @@
       </c>
       <c r="I387" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J387" s="2" t="inlineStr"/>
@@ -28263,7 +28263,7 @@
       </c>
       <c r="I423" s="2" t="inlineStr">
         <is>
-          <t>מזדמן</t>
+          <t>קבוע</t>
         </is>
       </c>
       <c r="J423" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Integrate 5 more IZ agreements; skip duplicate; idempotent seed loader
New single-page agreements: Mittman brothers (3 co-holders of avreich Zion Cohen),
Taubenfeld (2nd agreement, avreich Ordentlich), Yitzchak Hast (=Hast Itche),
Mendelson. Duplicate Yaakovzon file (already sent) is skipped. Donor names taken
from the agreements per instruction; set tier=יששכר־זבולון for holders that
weren't tagged (Hast, G. Mittman, Mendelson) so their box shows, and add the
avreich for the empty boxes. Seed file loader now clears only created='seed'
rows first, so re-seeds don't duplicate and user uploads are preserved.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhqHGEhN5Nq4zgX8f3S51z
</commit_message>
<xml_diff>
--- a/starter/crm-donors-filled.xlsx
+++ b/starter/crm-donors-filled.xlsx
@@ -11385,7 +11385,11 @@
           <t>דצמבר</t>
         </is>
       </c>
-      <c r="O166" s="2" t="inlineStr"/>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>יששכר_זבולון</t>
+        </is>
+      </c>
       <c r="P166" s="2" t="inlineStr"/>
       <c r="Q166" s="2" t="inlineStr">
         <is>
@@ -22469,7 +22473,11 @@
           <t>יולי</t>
         </is>
       </c>
-      <c r="O337" s="2" t="inlineStr"/>
+      <c r="O337" s="2" t="inlineStr">
+        <is>
+          <t>יששכר_זבולון</t>
+        </is>
+      </c>
       <c r="P337" s="2" t="inlineStr"/>
       <c r="Q337" s="2" t="inlineStr">
         <is>
@@ -23209,7 +23217,7 @@
       </c>
       <c r="O347" s="2" t="inlineStr">
         <is>
-          <t>קוויטל_כללי</t>
+          <t>יששכר_זבולון</t>
         </is>
       </c>
       <c r="P347" s="2" t="inlineStr">

</xml_diff>